<commit_message>
Add automatic Firebase Hosting deploy workflow on push to main
</commit_message>
<xml_diff>
--- a/reports/Selenium_Web_E2E_Test_Report.xlsx
+++ b/reports/Selenium_Web_E2E_Test_Report.xlsx
@@ -26,7 +26,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>8/3/2026, 9:42:50 AM</t>
+    <t>8/3/2026, 9:45:39 AM</t>
   </si>
   <si>
     <t>Total Test Cases Executed</t>
@@ -47,7 +47,7 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>172.82 seconds</t>
+    <t>172.58 seconds</t>
   </si>
   <si>
     <t>Suite Name</t>
@@ -92,7 +92,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>2026-08-03T04:10:27.103Z</t>
+    <t>2026-08-03T04:13:16.306Z</t>
   </si>
   <si>
     <t/>
@@ -110,7 +110,7 @@
     <t>Validation</t>
   </si>
   <si>
-    <t>2026-08-03T04:10:27.207Z</t>
+    <t>2026-08-03T04:13:16.419Z</t>
   </si>
   <si>
     <t>Empty email prompt handled</t>
@@ -122,7 +122,7 @@
     <t>Validate email without @ symbol format check</t>
   </si>
   <si>
-    <t>2026-08-03T04:10:37.407Z</t>
+    <t>2026-08-03T04:13:26.653Z</t>
   </si>
   <si>
     <t>Invalid email format caught</t>
@@ -134,7 +134,7 @@
     <t>Validate email without TLD format check</t>
   </si>
   <si>
-    <t>2026-08-03T04:10:47.572Z</t>
+    <t>2026-08-03T04:13:36.853Z</t>
   </si>
   <si>
     <t>Missing TLD handled</t>
@@ -146,7 +146,7 @@
     <t>Validate email with special characters in local part</t>
   </si>
   <si>
-    <t>2026-08-03T04:10:57.788Z</t>
+    <t>2026-08-03T04:13:47.035Z</t>
   </si>
   <si>
     <t>Tag sub-addressing accepted</t>
@@ -158,7 +158,7 @@
     <t>Validate short password error response (&lt;6 chars)</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:07.979Z</t>
+    <t>2026-08-03T04:13:57.242Z</t>
   </si>
   <si>
     <t>Min length password check passed</t>
@@ -170,7 +170,7 @@
     <t>Validate empty password field submission</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:08.094Z</t>
+    <t>2026-08-03T04:13:57.358Z</t>
   </si>
   <si>
     <t>Empty password check passed</t>
@@ -182,7 +182,7 @@
     <t>Validate password visibility toggle icon interaction</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:08.195Z</t>
+    <t>2026-08-03T04:13:57.475Z</t>
   </si>
   <si>
     <t>Password obscure state updated</t>
@@ -194,7 +194,7 @@
     <t>Validate Login / Register tab toggle switch</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:08.311Z</t>
+    <t>2026-08-03T04:13:57.591Z</t>
   </si>
   <si>
     <t>Switched to Register mode UI</t>
@@ -209,7 +209,7 @@
     <t>Functional</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:08.427Z</t>
+    <t>2026-08-03T04:13:57.708Z</t>
   </si>
   <si>
     <t>Full Name text input received</t>
@@ -221,7 +221,7 @@
     <t>Validate Register mode Phone Number input field</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:08.529Z</t>
+    <t>2026-08-03T04:13:57.824Z</t>
   </si>
   <si>
     <t>Phone Number text input received</t>
@@ -233,7 +233,7 @@
     <t>Validate valid credentials login submission payload</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:28.955Z</t>
+    <t>2026-08-03T04:14:18.174Z</t>
   </si>
   <si>
     <t>Auth payload sent to Supabase</t>
@@ -245,7 +245,7 @@
     <t>Validate forgot password link navigation trigger</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.058Z</t>
+    <t>2026-08-03T04:14:18.288Z</t>
   </si>
   <si>
     <t>Forgot password route triggered</t>
@@ -257,7 +257,7 @@
     <t>Validate reset password email input submission</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.174Z</t>
+    <t>2026-08-03T04:14:18.390Z</t>
   </si>
   <si>
     <t>Password recovery email dispatched</t>
@@ -269,7 +269,7 @@
     <t>Validate OTP verification screen load &amp; 6-digit pin boxes</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.277Z</t>
+    <t>2026-08-03T04:14:18.491Z</t>
   </si>
   <si>
     <t>OTP input boxes rendered</t>
@@ -281,7 +281,7 @@
     <t>Validate OTP submission with incomplete digits</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.392Z</t>
+    <t>2026-08-03T04:14:18.607Z</t>
   </si>
   <si>
     <t>Incomplete OTP prevented</t>
@@ -293,7 +293,7 @@
     <t>Validate OTP submission with valid 6-digit code</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.506Z</t>
+    <t>2026-08-03T04:14:18.719Z</t>
   </si>
   <si>
     <t>OTP verification confirmed</t>
@@ -305,7 +305,7 @@
     <t>Validate Onboarding screen slide 1 rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.608Z</t>
+    <t>2026-08-03T04:14:18.824Z</t>
   </si>
   <si>
     <t>Slide 1 hero image &amp; title visible</t>
@@ -317,7 +317,7 @@
     <t>Validate Onboarding screen slide 2 navigation swipe</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.709Z</t>
+    <t>2026-08-03T04:14:18.924Z</t>
   </si>
   <si>
     <t>Slide 2 posture tips displayed</t>
@@ -329,7 +329,7 @@
     <t>Validate Onboarding screen slide 3 navigation swipe</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.827Z</t>
+    <t>2026-08-03T04:14:19.041Z</t>
   </si>
   <si>
     <t>Slide 3 AI feature summary displayed</t>
@@ -341,7 +341,7 @@
     <t>Validate Onboarding Skip button action</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:29.940Z</t>
+    <t>2026-08-03T04:14:19.157Z</t>
   </si>
   <si>
     <t>Skipped onboarding to main screen</t>
@@ -353,7 +353,7 @@
     <t>Validate Onboarding Get Started button action</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.044Z</t>
+    <t>2026-08-03T04:14:19.273Z</t>
   </si>
   <si>
     <t>Completed onboarding flow</t>
@@ -365,7 +365,7 @@
     <t>Validate persistent login session token restoration</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.155Z</t>
+    <t>2026-08-03T04:14:19.373Z</t>
   </si>
   <si>
     <t>SharedPreferences session restored</t>
@@ -377,7 +377,7 @@
     <t>Validate auth error banner dismiss button</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.259Z</t>
+    <t>2026-08-03T04:14:19.474Z</t>
   </si>
   <si>
     <t>Error snackbar dismissed</t>
@@ -389,7 +389,7 @@
     <t>Validate whitespace trimming on email submission</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.374Z</t>
+    <t>2026-08-03T04:14:19.591Z</t>
   </si>
   <si>
     <t>Whitespace trimmed</t>
@@ -401,7 +401,7 @@
     <t>Validate registration password confirmation match</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.489Z</t>
+    <t>2026-08-03T04:14:19.705Z</t>
   </si>
   <si>
     <t>Passwords match verified</t>
@@ -413,7 +413,7 @@
     <t>Validate terms of service checkbox toggle</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.593Z</t>
+    <t>2026-08-03T04:14:19.806Z</t>
   </si>
   <si>
     <t>TOS checkbox toggled</t>
@@ -425,7 +425,7 @@
     <t>Validate privacy policy external link modal</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.709Z</t>
+    <t>2026-08-03T04:14:19.907Z</t>
   </si>
   <si>
     <t>Privacy policy displayed</t>
@@ -437,7 +437,7 @@
     <t>Validate logout button clearing local session state</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.823Z</t>
+    <t>2026-08-03T04:14:20.007Z</t>
   </si>
   <si>
     <t>Session storage cleared</t>
@@ -449,7 +449,7 @@
     <t>Validate redirect unauthenticated user to Login screen</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:30.927Z</t>
+    <t>2026-08-03T04:14:20.107Z</t>
   </si>
   <si>
     <t>Guarded route redirected to Login</t>
@@ -461,7 +461,7 @@
     <t>Validate remember me checkbox state persistence</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.042Z</t>
+    <t>2026-08-03T04:14:20.215Z</t>
   </si>
   <si>
     <t>Remember me checkbox state saved</t>
@@ -473,7 +473,7 @@
     <t>Validate google sign-in button option rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.143Z</t>
+    <t>2026-08-03T04:14:20.324Z</t>
   </si>
   <si>
     <t>Google OAuth button rendered</t>
@@ -485,7 +485,7 @@
     <t>Validate apple sign-in button option rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.257Z</t>
+    <t>2026-08-03T04:14:20.441Z</t>
   </si>
   <si>
     <t>Apple OAuth button rendered</t>
@@ -497,7 +497,7 @@
     <t>Validate session expiration popup prompt behavior</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.360Z</t>
+    <t>2026-08-03T04:14:20.557Z</t>
   </si>
   <si>
     <t>Session expiry popup displayed</t>
@@ -509,7 +509,7 @@
     <t>Validate auth token refresh background handler</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.477Z</t>
+    <t>2026-08-03T04:14:20.674Z</t>
   </si>
   <si>
     <t>Auth token refreshed</t>
@@ -524,7 +524,7 @@
     <t>Verify AppBar Title ConfidAI on Main Screen</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.577Z</t>
+    <t>2026-08-03T04:14:20.773Z</t>
   </si>
   <si>
     <t>AppBar title ConfidAI visible</t>
@@ -536,7 +536,7 @@
     <t>Verify Drawer Burger Icon opening navigation drawer</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.659Z</t>
+    <t>2026-08-03T04:14:20.857Z</t>
   </si>
   <si>
     <t>Navigation drawer opened</t>
@@ -548,7 +548,7 @@
     <t>Verify Drawer User Avatar rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.743Z</t>
+    <t>2026-08-03T04:14:20.940Z</t>
   </si>
   <si>
     <t>User Avatar circle visible in drawer header</t>
@@ -560,7 +560,7 @@
     <t>Verify Drawer User Name header label</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.825Z</t>
+    <t>2026-08-03T04:14:21.024Z</t>
   </si>
   <si>
     <t>User Name header rendered</t>
@@ -572,7 +572,7 @@
     <t>Verify Drawer item: Home menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:31.910Z</t>
+    <t>2026-08-03T04:14:21.105Z</t>
   </si>
   <si>
     <t>Home tab route active</t>
@@ -584,7 +584,7 @@
     <t>Verify Drawer item: History menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:41.995Z</t>
+    <t>2026-08-03T04:14:31.151Z</t>
   </si>
   <si>
     <t>Session History screen opened</t>
@@ -596,7 +596,7 @@
     <t>Verify Drawer item: Profile menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.062Z</t>
+    <t>2026-08-03T04:14:41.176Z</t>
   </si>
   <si>
     <t>Profile screen opened</t>
@@ -608,7 +608,7 @@
     <t>Verify Drawer item: Settings menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.152Z</t>
+    <t>2026-08-03T04:14:41.272Z</t>
   </si>
   <si>
     <t>Settings screen opened</t>
@@ -620,7 +620,7 @@
     <t>Verify Drawer item: Notifications menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.242Z</t>
+    <t>2026-08-03T04:14:41.356Z</t>
   </si>
   <si>
     <t>Notifications screen opened</t>
@@ -632,7 +632,7 @@
     <t>Verify Drawer item: Progress Report menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.325Z</t>
+    <t>2026-08-03T04:14:41.439Z</t>
   </si>
   <si>
     <t>Progress Report screen opened</t>
@@ -644,7 +644,7 @@
     <t>Verify Drawer item: Help &amp; Support menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.408Z</t>
+    <t>2026-08-03T04:14:41.523Z</t>
   </si>
   <si>
     <t>Help &amp; Support screen opened</t>
@@ -656,7 +656,7 @@
     <t>Verify Drawer item: About App menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.493Z</t>
+    <t>2026-08-03T04:14:41.606Z</t>
   </si>
   <si>
     <t>About App screen opened</t>
@@ -668,7 +668,7 @@
     <t>Verify Drawer item: Tips Library menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.593Z</t>
+    <t>2026-08-03T04:14:41.690Z</t>
   </si>
   <si>
     <t>Tips Library screen opened</t>
@@ -680,7 +680,7 @@
     <t>Verify Drawer item: Achievements menu item click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.674Z</t>
+    <t>2026-08-03T04:14:41.773Z</t>
   </si>
   <si>
     <t>Achievements screen opened</t>
@@ -692,7 +692,7 @@
     <t>Verify Settings screen: Blue Accent Color swatch selection</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.759Z</t>
+    <t>2026-08-03T04:14:41.856Z</t>
   </si>
   <si>
     <t>Theme accent set to Ocean Blue</t>
@@ -704,7 +704,7 @@
     <t>Verify Settings screen: Orange Accent Color swatch selection</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.842Z</t>
+    <t>2026-08-03T04:14:41.939Z</t>
   </si>
   <si>
     <t>Theme accent set to Sunset Orange</t>
@@ -716,7 +716,7 @@
     <t>Verify Settings screen: Green Accent Color swatch selection</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:52.926Z</t>
+    <t>2026-08-03T04:14:42.022Z</t>
   </si>
   <si>
     <t>Theme accent set to Forest Green</t>
@@ -728,7 +728,7 @@
     <t>Verify Settings screen: Dark Mode Switch toggle ON</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.009Z</t>
+    <t>2026-08-03T04:14:42.106Z</t>
   </si>
   <si>
     <t>Dark mode theme activated</t>
@@ -740,7 +740,7 @@
     <t>Verify Settings screen: Dark Mode Switch toggle OFF</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.092Z</t>
+    <t>2026-08-03T04:14:42.190Z</t>
   </si>
   <si>
     <t>Light mode theme activated</t>
@@ -752,7 +752,7 @@
     <t>Verify Edit Profile screen load &amp; form text controllers</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.174Z</t>
+    <t>2026-08-03T04:14:42.272Z</t>
   </si>
   <si>
     <t>Profile name &amp; bio input fields editable</t>
@@ -764,7 +764,7 @@
     <t>Verify Edit Profile save changes button trigger</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.259Z</t>
+    <t>2026-08-03T04:14:42.356Z</t>
   </si>
   <si>
     <t>Profile changes saved to SharedPreferences</t>
@@ -776,7 +776,7 @@
     <t>Verify Notifications screen recent notification list items</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.343Z</t>
+    <t>2026-08-03T04:14:42.439Z</t>
   </si>
   <si>
     <t>5 notification card items rendered</t>
@@ -788,7 +788,7 @@
     <t>Verify Progress Report screen 28-day streak calendar grid</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.425Z</t>
+    <t>2026-08-03T04:14:42.521Z</t>
   </si>
   <si>
     <t>Streak calendar 28 day circles rendered</t>
@@ -800,7 +800,7 @@
     <t>Verify Achievements screen unlocked badge icons</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.510Z</t>
+    <t>2026-08-03T04:14:42.605Z</t>
   </si>
   <si>
     <t>Achievement badge list displayed</t>
@@ -812,7 +812,7 @@
     <t>Verify Tips Library card expansion details</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.593Z</t>
+    <t>2026-08-03T04:14:42.689Z</t>
   </si>
   <si>
     <t>Body language tip detail card expanded</t>
@@ -824,7 +824,7 @@
     <t>Verify Help &amp; Support FAQ accordion expansion</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.675Z</t>
+    <t>2026-08-03T04:14:42.773Z</t>
   </si>
   <si>
     <t>FAQ answer text expanded</t>
@@ -836,7 +836,7 @@
     <t>Verify About App version string &amp; tech stack overview</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.759Z</t>
+    <t>2026-08-03T04:14:42.856Z</t>
   </si>
   <si>
     <t>App version 1.0.0 &amp; Flutter framework credited</t>
@@ -848,7 +848,7 @@
     <t>Verify Bottom Navigation Bar Home tab icon click</t>
   </si>
   <si>
-    <t>2026-08-03T04:11:53.842Z</t>
+    <t>2026-08-03T04:14:42.938Z</t>
   </si>
   <si>
     <t>Switched to Home tab</t>
@@ -860,7 +860,7 @@
     <t>Verify Bottom Navigation Bar History tab icon click</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:03.944Z</t>
+    <t>2026-08-03T04:14:52.986Z</t>
   </si>
   <si>
     <t>Switched to History tab</t>
@@ -872,7 +872,7 @@
     <t>Verify Bottom Navigation Bar Profile tab icon click</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:13.987Z</t>
+    <t>2026-08-03T04:15:03.048Z</t>
   </si>
   <si>
     <t>Switched to Profile tab</t>
@@ -884,7 +884,7 @@
     <t>Verify Bottom Navigation Bar Settings tab icon click</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:14.080Z</t>
+    <t>2026-08-03T04:15:03.143Z</t>
   </si>
   <si>
     <t>Switched to Settings tab</t>
@@ -896,7 +896,7 @@
     <t>Verify App Bar back button navigation stack pop</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:14.163Z</t>
+    <t>2026-08-03T04:15:03.225Z</t>
   </si>
   <si>
     <t>Back button popped route stack</t>
@@ -908,7 +908,7 @@
     <t>Verify Deep linking route resolution for /history path</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:14.247Z</t>
+    <t>2026-08-03T04:15:03.310Z</t>
   </si>
   <si>
     <t>Direct URL /history resolved</t>
@@ -920,7 +920,7 @@
     <t>Verify Deep linking route resolution for /settings path</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:14.331Z</t>
+    <t>2026-08-03T04:15:03.394Z</t>
   </si>
   <si>
     <t>Direct URL /settings resolved</t>
@@ -932,7 +932,7 @@
     <t>Verify 404 Page Not Found route fallback screen</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:14.414Z</t>
+    <t>2026-08-03T04:15:03.477Z</t>
   </si>
   <si>
     <t>Fallback 404 route rendered</t>
@@ -947,7 +947,7 @@
     <t>Verify Start Practice Session button on Home Screen</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:24.486Z</t>
+    <t>2026-08-03T04:15:13.550Z</t>
   </si>
   <si>
     <t>Start Practice Session button active</t>
@@ -959,7 +959,7 @@
     <t>Verify Camera permission dialog auto-grant via fake UI flags</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:24.613Z</t>
+    <t>2026-08-03T04:15:13.675Z</t>
   </si>
   <si>
     <t>Fake media device flags granted video stream</t>
@@ -971,7 +971,7 @@
     <t>Verify Y4M real sample video stream feed injection (--use-file-for-fake-video-capture)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:24.744Z</t>
+    <t>2026-08-03T04:15:13.812Z</t>
   </si>
   <si>
     <t>sample_video.y4m video stream feeding HTML5 video element</t>
@@ -983,7 +983,7 @@
     <t>Verify Camera preview widget initialization &amp; aspect ratio container</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:24.880Z</t>
+    <t>2026-08-03T04:15:13.940Z</t>
   </si>
   <si>
     <t>Camera view container initialized</t>
@@ -995,7 +995,7 @@
     <t>Verify Live recording duration timer start (00:00 count up)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:25.013Z</t>
+    <t>2026-08-03T04:15:14.063Z</t>
   </si>
   <si>
     <t>Timer counter incrementing</t>
@@ -1007,7 +1007,7 @@
     <t>Verify Floating Record / Pause control button rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:25.146Z</t>
+    <t>2026-08-03T04:15:14.189Z</t>
   </si>
   <si>
     <t>Floating record button visible</t>
@@ -1019,7 +1019,7 @@
     <t>Verify Live Posture Score indicator widget on overlay</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:25.280Z</t>
+    <t>2026-08-03T04:15:14.309Z</t>
   </si>
   <si>
     <t>Live posture score overlay active</t>
@@ -1031,7 +1031,7 @@
     <t>Verify Live Head Stability gauge on camera view overlay</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:25.412Z</t>
+    <t>2026-08-03T04:15:14.442Z</t>
   </si>
   <si>
     <t>Head stability gauge active</t>
@@ -1043,7 +1043,7 @@
     <t>Verify Live Gesture detection feedback indicator</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:25.547Z</t>
+    <t>2026-08-03T04:15:14.576Z</t>
   </si>
   <si>
     <t>Gesture detection indicator active</t>
@@ -1055,7 +1055,7 @@
     <t>Verify Stop Session button action &amp; session finalization</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:45.674Z</t>
+    <t>2026-08-03T04:15:34.717Z</t>
   </si>
   <si>
     <t>Recording stopped and video buffered</t>
@@ -1067,7 +1067,7 @@
     <t>Verify AI Analysis pipeline payload dispatch to Render backend</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:45.796Z</t>
+    <t>2026-08-03T04:15:34.840Z</t>
   </si>
   <si>
     <t>Video payload sent to AI backend service</t>
@@ -1079,7 +1079,7 @@
     <t>Verify Results Screen transition after analysis completion</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:45.929Z</t>
+    <t>2026-08-03T04:15:34.971Z</t>
   </si>
   <si>
     <t>Navigated to Results Screen</t>
@@ -1091,7 +1091,7 @@
     <t>Verify Overall Confidence Score gauge rendering (0-100%)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.062Z</t>
+    <t>2026-08-03T04:15:35.106Z</t>
   </si>
   <si>
     <t>Overall score gauge displayed</t>
@@ -1103,7 +1103,7 @@
     <t>Verify Posture Sub-Score card breakdown (40% weight)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.195Z</t>
+    <t>2026-08-03T04:15:35.241Z</t>
   </si>
   <si>
     <t>Posture sub-score breakdown visible</t>
@@ -1115,7 +1115,7 @@
     <t>Verify Head Stability Sub-Score card breakdown (30% weight)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.329Z</t>
+    <t>2026-08-03T04:15:35.372Z</t>
   </si>
   <si>
     <t>Head stability sub-score breakdown visible</t>
@@ -1127,7 +1127,7 @@
     <t>Verify Gesture Activity Sub-Score card breakdown (30% weight)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.462Z</t>
+    <t>2026-08-03T04:15:35.506Z</t>
   </si>
   <si>
     <t>Gesture sub-score breakdown visible</t>
@@ -1139,7 +1139,7 @@
     <t>Verify Key Improvement Recommendations list</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.596Z</t>
+    <t>2026-08-03T04:15:35.635Z</t>
   </si>
   <si>
     <t>AI feedback recommendations list populated</t>
@@ -1151,7 +1151,7 @@
     <t>Verify Save Session to History SharedPreferences database</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.729Z</t>
+    <t>2026-08-03T04:15:35.757Z</t>
   </si>
   <si>
     <t>Session JSON record committed to SharedPreferences</t>
@@ -1163,7 +1163,7 @@
     <t>Verify Export Session Report CSV button click action</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.862Z</t>
+    <t>2026-08-03T04:15:35.887Z</t>
   </si>
   <si>
     <t>CSV file export triggered via Share API</t>
@@ -1175,7 +1175,7 @@
     <t>Verify Export Session Summary PDF document generation</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:46.995Z</t>
+    <t>2026-08-03T04:15:36.008Z</t>
   </si>
   <si>
     <t>PDF document compiled via printing package</t>
@@ -1187,7 +1187,7 @@
     <t>Verify Session History log list updated with new session item</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:47.129Z</t>
+    <t>2026-08-03T04:15:36.140Z</t>
   </si>
   <si>
     <t>History list contains newly completed session</t>
@@ -1199,7 +1199,7 @@
     <t>Verify Session History item score pill color coding (Green/Orange)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:47.262Z</t>
+    <t>2026-08-03T04:15:36.274Z</t>
   </si>
   <si>
     <t>Score pill color matches performance tier</t>
@@ -1211,7 +1211,7 @@
     <t>Verify Session History Compare Last 2 Sessions modal trigger</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:47.395Z</t>
+    <t>2026-08-03T04:15:36.409Z</t>
   </si>
   <si>
     <t>Compare modal bottom sheet opened</t>
@@ -1223,7 +1223,7 @@
     <t>Verify Session Comparison metric deltas (+/- % diff calculations)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:47.529Z</t>
+    <t>2026-08-03T04:15:36.543Z</t>
   </si>
   <si>
     <t>Posture/head/gesture diff metrics accurate</t>
@@ -1235,7 +1235,7 @@
     <t>Verify Clear Session History confirmation dialog</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:47.660Z</t>
+    <t>2026-08-03T04:15:36.676Z</t>
   </si>
   <si>
     <t>Clear history dialog prompted</t>
@@ -1247,7 +1247,7 @@
     <t>Verify Cancel Camera Session return to Home screen</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:47.796Z</t>
+    <t>2026-08-03T04:15:36.809Z</t>
   </si>
   <si>
     <t>Session cancelled cleanly</t>
@@ -1259,7 +1259,7 @@
     <t>Verify Retry Analysis button action on backend failure</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:47.929Z</t>
+    <t>2026-08-03T04:15:36.942Z</t>
   </si>
   <si>
     <t>Retry analysis request dispatched</t>
@@ -1271,7 +1271,7 @@
     <t>Verify Practice Reminder notification trigger logic</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.062Z</t>
+    <t>2026-08-03T04:15:37.069Z</t>
   </si>
   <si>
     <t>Weekly practice reminder scheduled</t>
@@ -1283,7 +1283,7 @@
     <t>Verify Streak counter increment after session completion</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.194Z</t>
+    <t>2026-08-03T04:15:37.192Z</t>
   </si>
   <si>
     <t>Streak count updated in calendar</t>
@@ -1295,7 +1295,7 @@
     <t>Verify Achievement unlock detection after 3 completed sessions</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.326Z</t>
+    <t>2026-08-03T04:15:37.324Z</t>
   </si>
   <si>
     <t>3-session achievement unlocked</t>
@@ -1307,7 +1307,7 @@
     <t>Verify Audio waveform feedback visualizer during recording</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.462Z</t>
+    <t>2026-08-03T04:15:37.448Z</t>
   </si>
   <si>
     <t>Audio visualizer active</t>
@@ -1319,7 +1319,7 @@
     <t>Verify Camera device switch toggle action (front/back lens)</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.596Z</t>
+    <t>2026-08-03T04:15:37.571Z</t>
   </si>
   <si>
     <t>Lens toggled</t>
@@ -1331,7 +1331,7 @@
     <t>Verify Low-light environment warning prompt banner</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.729Z</t>
+    <t>2026-08-03T04:15:37.695Z</t>
   </si>
   <si>
     <t>Low-light prompt displayed</t>
@@ -1343,7 +1343,7 @@
     <t>Verify AI posture angle breakdown graph component</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.862Z</t>
+    <t>2026-08-03T04:15:37.829Z</t>
   </si>
   <si>
     <t>Angle chart rendered</t>
@@ -1355,7 +1355,7 @@
     <t>Verify Real-time feedback overlay toggle ON/OFF setting</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:48.996Z</t>
+    <t>2026-08-03T04:15:37.950Z</t>
   </si>
   <si>
     <t>Feedback overlay toggled</t>
@@ -1370,7 +1370,7 @@
     <t>Verify responsive layout adaptation at 1280x800 desktop resolution</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.062Z</t>
+    <t>2026-08-03T04:15:38.018Z</t>
   </si>
   <si>
     <t>Desktop layout verified</t>
@@ -1382,7 +1382,7 @@
     <t>Verify responsive layout adaptation at 768x1024 tablet resolution</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.128Z</t>
+    <t>2026-08-03T04:15:38.094Z</t>
   </si>
   <si>
     <t>Tablet layout verified</t>
@@ -1394,7 +1394,7 @@
     <t>Verify responsive layout adaptation at 375x812 mobile screen size</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.193Z</t>
+    <t>2026-08-03T04:15:38.156Z</t>
   </si>
   <si>
     <t>Mobile viewport layout verified</t>
@@ -1406,7 +1406,7 @@
     <t>Verify Flutter web semantics tree accessibility node rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.262Z</t>
+    <t>2026-08-03T04:15:38.230Z</t>
   </si>
   <si>
     <t>flt-semantics nodes active</t>
@@ -1418,7 +1418,7 @@
     <t>Verify ARIA accessibility labels for screen reader compatibility</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.329Z</t>
+    <t>2026-08-03T04:15:38.305Z</t>
   </si>
   <si>
     <t>ARIA labels present on key controls</t>
@@ -1430,7 +1430,7 @@
     <t>Verify color contrast accessibility ratio for text elements</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.396Z</t>
+    <t>2026-08-03T04:15:38.373Z</t>
   </si>
   <si>
     <t>WCAG AAA contrast verified</t>
@@ -1442,7 +1442,7 @@
     <t>Verify font scaling and typography hierarchy readability</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.462Z</t>
+    <t>2026-08-03T04:15:38.439Z</t>
   </si>
   <si>
     <t>Google Inter font scale validated</t>
@@ -1454,7 +1454,7 @@
     <t>Verify glassmorphism card elevation and shadow rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.529Z</t>
+    <t>2026-08-03T04:15:38.505Z</t>
   </si>
   <si>
     <t>Box shadows rendered smoothly</t>
@@ -1466,7 +1466,7 @@
     <t>Verify dynamic gradient background rendering in light mode</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.596Z</t>
+    <t>2026-08-03T04:15:38.573Z</t>
   </si>
   <si>
     <t>Light mode gradient active</t>
@@ -1478,7 +1478,7 @@
     <t>Verify dynamic dark mode background palette transitions</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.662Z</t>
+    <t>2026-08-03T04:15:38.640Z</t>
   </si>
   <si>
     <t>Dark mode palette active</t>
@@ -1490,7 +1490,7 @@
     <t>Verify micro-animation smooth transition on button hover</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.728Z</t>
+    <t>2026-08-03T04:15:38.710Z</t>
   </si>
   <si>
     <t>Hover animations active</t>
@@ -1502,7 +1502,7 @@
     <t>Verify modal backdrop blur effect rendering</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.795Z</t>
+    <t>2026-08-03T04:15:38.775Z</t>
   </si>
   <si>
     <t>Backdrop blur filter applied</t>
@@ -1514,7 +1514,7 @@
     <t>Verify icon set rendering consistency across screens</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.862Z</t>
+    <t>2026-08-03T04:15:38.840Z</t>
   </si>
   <si>
     <t>Material Icons rendered</t>
@@ -1526,7 +1526,7 @@
     <t>Verify keyboard navigation tab focus ring visibility</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.929Z</t>
+    <t>2026-08-03T04:15:38.909Z</t>
   </si>
   <si>
     <t>Tab index focus indicators active</t>
@@ -1538,7 +1538,7 @@
     <t>Verify screen reader announcements on state change</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:49.995Z</t>
+    <t>2026-08-03T04:15:38.979Z</t>
   </si>
   <si>
     <t>Live region announcements triggered</t>
@@ -1550,7 +1550,7 @@
     <t>Verify custom scrollbar styling and smooth scrolling</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:50.062Z</t>
+    <t>2026-08-03T04:15:39.055Z</t>
   </si>
   <si>
     <t>Smooth scrolling operational</t>
@@ -1562,7 +1562,7 @@
     <t>Verify high-contrast high-visibility mode toggle</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:50.129Z</t>
+    <t>2026-08-03T04:15:39.130Z</t>
   </si>
   <si>
     <t>High-contrast mode supported</t>
@@ -1574,7 +1574,7 @@
     <t>Verify loading skeleton placeholders during web asset fetch</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:50.190Z</t>
+    <t>2026-08-03T04:15:39.191Z</t>
   </si>
   <si>
     <t>Skeleton loaders displayed</t>
@@ -1586,7 +1586,7 @@
     <t>Verify tooltip popover hover display on metric cards</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:50.262Z</t>
+    <t>2026-08-03T04:15:39.260Z</t>
   </si>
   <si>
     <t>Tooltip popovers active</t>
@@ -1598,7 +1598,7 @@
     <t>Verify smooth page transition route animations</t>
   </si>
   <si>
-    <t>2026-08-03T04:12:50.329Z</t>
+    <t>2026-08-03T04:15:39.330Z</t>
   </si>
   <si>
     <t>Route transitions smooth</t>
@@ -2179,7 +2179,7 @@
         <v>25</v>
       </c>
       <c r="F2">
-        <v>14791</v>
+        <v>14755</v>
       </c>
       <c r="G2" t="s">
         <v>26</v>
@@ -2208,7 +2208,7 @@
         <v>25</v>
       </c>
       <c r="F3">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="G3" t="s">
         <v>32</v>
@@ -2237,7 +2237,7 @@
         <v>25</v>
       </c>
       <c r="F4">
-        <v>10320</v>
+        <v>10354</v>
       </c>
       <c r="G4" t="s">
         <v>36</v>
@@ -2266,7 +2266,7 @@
         <v>25</v>
       </c>
       <c r="F5">
-        <v>10284</v>
+        <v>10320</v>
       </c>
       <c r="G5" t="s">
         <v>40</v>
@@ -2295,7 +2295,7 @@
         <v>25</v>
       </c>
       <c r="F6">
-        <v>10336</v>
+        <v>10302</v>
       </c>
       <c r="G6" t="s">
         <v>44</v>
@@ -2324,7 +2324,7 @@
         <v>25</v>
       </c>
       <c r="F7">
-        <v>10310</v>
+        <v>10326</v>
       </c>
       <c r="G7" t="s">
         <v>48</v>
@@ -2353,7 +2353,7 @@
         <v>25</v>
       </c>
       <c r="F8">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G8" t="s">
         <v>52</v>
@@ -2382,7 +2382,7 @@
         <v>25</v>
       </c>
       <c r="F9">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="G9" t="s">
         <v>56</v>
@@ -2469,7 +2469,7 @@
         <v>25</v>
       </c>
       <c r="F12">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="G12" t="s">
         <v>69</v>
@@ -2498,7 +2498,7 @@
         <v>25</v>
       </c>
       <c r="F13">
-        <v>20546</v>
+        <v>20469</v>
       </c>
       <c r="G13" t="s">
         <v>73</v>
@@ -2527,7 +2527,7 @@
         <v>25</v>
       </c>
       <c r="F14">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="G14" t="s">
         <v>77</v>
@@ -2556,7 +2556,7 @@
         <v>25</v>
       </c>
       <c r="F15">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="G15" t="s">
         <v>81</v>
@@ -2585,7 +2585,7 @@
         <v>25</v>
       </c>
       <c r="F16">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="G16" t="s">
         <v>85</v>
@@ -2614,7 +2614,7 @@
         <v>25</v>
       </c>
       <c r="F17">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G17" t="s">
         <v>89</v>
@@ -2643,7 +2643,7 @@
         <v>25</v>
       </c>
       <c r="F18">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G18" t="s">
         <v>93</v>
@@ -2672,7 +2672,7 @@
         <v>25</v>
       </c>
       <c r="F19">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G19" t="s">
         <v>97</v>
@@ -2701,7 +2701,7 @@
         <v>25</v>
       </c>
       <c r="F20">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G20" t="s">
         <v>101</v>
@@ -2759,7 +2759,7 @@
         <v>25</v>
       </c>
       <c r="F22">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="G22" t="s">
         <v>109</v>
@@ -2788,7 +2788,7 @@
         <v>25</v>
       </c>
       <c r="F23">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="G23" t="s">
         <v>113</v>
@@ -2817,7 +2817,7 @@
         <v>25</v>
       </c>
       <c r="F24">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="G24" t="s">
         <v>117</v>
@@ -2846,7 +2846,7 @@
         <v>25</v>
       </c>
       <c r="F25">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="G25" t="s">
         <v>121</v>
@@ -2875,7 +2875,7 @@
         <v>25</v>
       </c>
       <c r="F26">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G26" t="s">
         <v>125</v>
@@ -2904,7 +2904,7 @@
         <v>25</v>
       </c>
       <c r="F27">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G27" t="s">
         <v>129</v>
@@ -2933,7 +2933,7 @@
         <v>25</v>
       </c>
       <c r="F28">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="G28" t="s">
         <v>133</v>
@@ -2962,7 +2962,7 @@
         <v>25</v>
       </c>
       <c r="F29">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="G29" t="s">
         <v>137</v>
@@ -2991,7 +2991,7 @@
         <v>25</v>
       </c>
       <c r="F30">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="G30" t="s">
         <v>141</v>
@@ -3020,7 +3020,7 @@
         <v>25</v>
       </c>
       <c r="F31">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="G31" t="s">
         <v>145</v>
@@ -3049,7 +3049,7 @@
         <v>25</v>
       </c>
       <c r="F32">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="G32" t="s">
         <v>149</v>
@@ -3078,7 +3078,7 @@
         <v>25</v>
       </c>
       <c r="F33">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="G33" t="s">
         <v>153</v>
@@ -3107,7 +3107,7 @@
         <v>25</v>
       </c>
       <c r="F34">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="G34" t="s">
         <v>157</v>
@@ -3136,7 +3136,7 @@
         <v>25</v>
       </c>
       <c r="F35">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="G35" t="s">
         <v>161</v>
@@ -3165,7 +3165,7 @@
         <v>25</v>
       </c>
       <c r="F36">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G36" t="s">
         <v>165</v>
@@ -3194,7 +3194,7 @@
         <v>25</v>
       </c>
       <c r="F37">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="G37" t="s">
         <v>170</v>
@@ -3223,7 +3223,7 @@
         <v>25</v>
       </c>
       <c r="F38">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G38" t="s">
         <v>174</v>
@@ -3252,7 +3252,7 @@
         <v>25</v>
       </c>
       <c r="F39">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G39" t="s">
         <v>178</v>
@@ -3281,7 +3281,7 @@
         <v>25</v>
       </c>
       <c r="F40">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G40" t="s">
         <v>182</v>
@@ -3310,7 +3310,7 @@
         <v>25</v>
       </c>
       <c r="F41">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="G41" t="s">
         <v>186</v>
@@ -3339,7 +3339,7 @@
         <v>25</v>
       </c>
       <c r="F42">
-        <v>10185</v>
+        <v>10146</v>
       </c>
       <c r="G42" t="s">
         <v>190</v>
@@ -3368,7 +3368,7 @@
         <v>25</v>
       </c>
       <c r="F43">
-        <v>10167</v>
+        <v>10125</v>
       </c>
       <c r="G43" t="s">
         <v>194</v>
@@ -3397,7 +3397,7 @@
         <v>25</v>
       </c>
       <c r="F44">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="G44" t="s">
         <v>198</v>
@@ -3426,7 +3426,7 @@
         <v>25</v>
       </c>
       <c r="F45">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="G45" t="s">
         <v>202</v>
@@ -3455,7 +3455,7 @@
         <v>25</v>
       </c>
       <c r="F46">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G46" t="s">
         <v>206</v>
@@ -3513,7 +3513,7 @@
         <v>25</v>
       </c>
       <c r="F48">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G48" t="s">
         <v>214</v>
@@ -3542,7 +3542,7 @@
         <v>25</v>
       </c>
       <c r="F49">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="G49" t="s">
         <v>218</v>
@@ -3571,7 +3571,7 @@
         <v>25</v>
       </c>
       <c r="F50">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G50" t="s">
         <v>222</v>
@@ -3600,7 +3600,7 @@
         <v>25</v>
       </c>
       <c r="F51">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G51" t="s">
         <v>226</v>
@@ -3658,7 +3658,7 @@
         <v>25</v>
       </c>
       <c r="F53">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G53" t="s">
         <v>234</v>
@@ -3687,7 +3687,7 @@
         <v>25</v>
       </c>
       <c r="F54">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G54" t="s">
         <v>238</v>
@@ -3716,7 +3716,7 @@
         <v>25</v>
       </c>
       <c r="F55">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G55" t="s">
         <v>242</v>
@@ -3774,7 +3774,7 @@
         <v>25</v>
       </c>
       <c r="F57">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G57" t="s">
         <v>250</v>
@@ -3803,7 +3803,7 @@
         <v>25</v>
       </c>
       <c r="F58">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G58" t="s">
         <v>254</v>
@@ -3832,7 +3832,7 @@
         <v>25</v>
       </c>
       <c r="F59">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G59" t="s">
         <v>258</v>
@@ -3861,7 +3861,7 @@
         <v>25</v>
       </c>
       <c r="F60">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G60" t="s">
         <v>262</v>
@@ -3919,7 +3919,7 @@
         <v>25</v>
       </c>
       <c r="F62">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G62" t="s">
         <v>270</v>
@@ -3948,7 +3948,7 @@
         <v>25</v>
       </c>
       <c r="F63">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G63" t="s">
         <v>274</v>
@@ -3977,7 +3977,7 @@
         <v>25</v>
       </c>
       <c r="F64">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G64" t="s">
         <v>278</v>
@@ -4006,7 +4006,7 @@
         <v>25</v>
       </c>
       <c r="F65">
-        <v>10201</v>
+        <v>10148</v>
       </c>
       <c r="G65" t="s">
         <v>282</v>
@@ -4035,7 +4035,7 @@
         <v>25</v>
       </c>
       <c r="F66">
-        <v>10143</v>
+        <v>10162</v>
       </c>
       <c r="G66" t="s">
         <v>286</v>
@@ -4064,7 +4064,7 @@
         <v>25</v>
       </c>
       <c r="F67">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G67" t="s">
         <v>290</v>
@@ -4093,7 +4093,7 @@
         <v>25</v>
       </c>
       <c r="F68">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G68" t="s">
         <v>294</v>
@@ -4122,7 +4122,7 @@
         <v>25</v>
       </c>
       <c r="F69">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G69" t="s">
         <v>298</v>
@@ -4151,7 +4151,7 @@
         <v>25</v>
       </c>
       <c r="F70">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G70" t="s">
         <v>302</v>
@@ -4238,7 +4238,7 @@
         <v>25</v>
       </c>
       <c r="F73">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="G73" t="s">
         <v>315</v>
@@ -4267,7 +4267,7 @@
         <v>25</v>
       </c>
       <c r="F74">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="G74" t="s">
         <v>319</v>
@@ -4296,7 +4296,7 @@
         <v>25</v>
       </c>
       <c r="F75">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G75" t="s">
         <v>323</v>
@@ -4325,7 +4325,7 @@
         <v>25</v>
       </c>
       <c r="F76">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="G76" t="s">
         <v>327</v>
@@ -4354,7 +4354,7 @@
         <v>25</v>
       </c>
       <c r="F77">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="G77" t="s">
         <v>331</v>
@@ -4383,7 +4383,7 @@
         <v>25</v>
       </c>
       <c r="F78">
-        <v>283</v>
+        <v>270</v>
       </c>
       <c r="G78" t="s">
         <v>335</v>
@@ -4441,7 +4441,7 @@
         <v>25</v>
       </c>
       <c r="F80">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G80" t="s">
         <v>343</v>
@@ -4470,7 +4470,7 @@
         <v>25</v>
       </c>
       <c r="F81">
-        <v>20277</v>
+        <v>20291</v>
       </c>
       <c r="G81" t="s">
         <v>347</v>
@@ -4499,7 +4499,7 @@
         <v>25</v>
       </c>
       <c r="F82">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G82" t="s">
         <v>351</v>
@@ -4528,7 +4528,7 @@
         <v>25</v>
       </c>
       <c r="F83">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G83" t="s">
         <v>355</v>
@@ -4557,7 +4557,7 @@
         <v>25</v>
       </c>
       <c r="F84">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="G84" t="s">
         <v>359</v>
@@ -4586,7 +4586,7 @@
         <v>25</v>
       </c>
       <c r="F85">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="G85" t="s">
         <v>363</v>
@@ -4615,7 +4615,7 @@
         <v>25</v>
       </c>
       <c r="F86">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G86" t="s">
         <v>367</v>
@@ -4644,7 +4644,7 @@
         <v>25</v>
       </c>
       <c r="F87">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G87" t="s">
         <v>371</v>
@@ -4673,7 +4673,7 @@
         <v>25</v>
       </c>
       <c r="F88">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="G88" t="s">
         <v>375</v>
@@ -4702,7 +4702,7 @@
         <v>25</v>
       </c>
       <c r="F89">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="G89" t="s">
         <v>379</v>
@@ -4731,7 +4731,7 @@
         <v>25</v>
       </c>
       <c r="F90">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="G90" t="s">
         <v>383</v>
@@ -4760,7 +4760,7 @@
         <v>25</v>
       </c>
       <c r="F91">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="G91" t="s">
         <v>387</v>
@@ -4789,7 +4789,7 @@
         <v>25</v>
       </c>
       <c r="F92">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G92" t="s">
         <v>391</v>
@@ -4847,7 +4847,7 @@
         <v>25</v>
       </c>
       <c r="F94">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="G94" t="s">
         <v>399</v>
@@ -4876,7 +4876,7 @@
         <v>25</v>
       </c>
       <c r="F95">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G95" t="s">
         <v>403</v>
@@ -4905,7 +4905,7 @@
         <v>25</v>
       </c>
       <c r="F96">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G96" t="s">
         <v>407</v>
@@ -4934,7 +4934,7 @@
         <v>25</v>
       </c>
       <c r="F97">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="G97" t="s">
         <v>411</v>
@@ -4963,7 +4963,7 @@
         <v>25</v>
       </c>
       <c r="F98">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G98" t="s">
         <v>415</v>
@@ -4992,7 +4992,7 @@
         <v>25</v>
       </c>
       <c r="F99">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="G99" t="s">
         <v>419</v>
@@ -5021,7 +5021,7 @@
         <v>25</v>
       </c>
       <c r="F100">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="G100" t="s">
         <v>423</v>
@@ -5079,7 +5079,7 @@
         <v>25</v>
       </c>
       <c r="F102">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="G102" t="s">
         <v>431</v>
@@ -5108,7 +5108,7 @@
         <v>25</v>
       </c>
       <c r="F103">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="G103" t="s">
         <v>435</v>
@@ -5137,7 +5137,7 @@
         <v>25</v>
       </c>
       <c r="F104">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="G104" t="s">
         <v>439</v>
@@ -5166,7 +5166,7 @@
         <v>25</v>
       </c>
       <c r="F105">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G105" t="s">
         <v>443</v>
@@ -5195,7 +5195,7 @@
         <v>25</v>
       </c>
       <c r="F106">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="G106" t="s">
         <v>447</v>
@@ -5224,7 +5224,7 @@
         <v>25</v>
       </c>
       <c r="F107">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G107" t="s">
         <v>452</v>
@@ -5253,7 +5253,7 @@
         <v>25</v>
       </c>
       <c r="F108">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="G108" t="s">
         <v>456</v>
@@ -5282,7 +5282,7 @@
         <v>25</v>
       </c>
       <c r="F109">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G109" t="s">
         <v>460</v>
@@ -5311,7 +5311,7 @@
         <v>25</v>
       </c>
       <c r="F110">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="G110" t="s">
         <v>464</v>
@@ -5340,7 +5340,7 @@
         <v>25</v>
       </c>
       <c r="F111">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="G111" t="s">
         <v>468</v>
@@ -5369,7 +5369,7 @@
         <v>25</v>
       </c>
       <c r="F112">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G112" t="s">
         <v>472</v>
@@ -5427,7 +5427,7 @@
         <v>25</v>
       </c>
       <c r="F114">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G114" t="s">
         <v>480</v>
@@ -5514,7 +5514,7 @@
         <v>25</v>
       </c>
       <c r="F117">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="G117" t="s">
         <v>492</v>
@@ -5543,7 +5543,7 @@
         <v>25</v>
       </c>
       <c r="F118">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G118" t="s">
         <v>496</v>
@@ -5572,7 +5572,7 @@
         <v>25</v>
       </c>
       <c r="F119">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G119" t="s">
         <v>500</v>
@@ -5601,7 +5601,7 @@
         <v>25</v>
       </c>
       <c r="F120">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G120" t="s">
         <v>504</v>
@@ -5630,7 +5630,7 @@
         <v>25</v>
       </c>
       <c r="F121">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G121" t="s">
         <v>508</v>
@@ -5659,7 +5659,7 @@
         <v>25</v>
       </c>
       <c r="F122">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="G122" t="s">
         <v>512</v>
@@ -5688,7 +5688,7 @@
         <v>25</v>
       </c>
       <c r="F123">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="G123" t="s">
         <v>516</v>
@@ -5746,7 +5746,7 @@
         <v>25</v>
       </c>
       <c r="F125">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="G125" t="s">
         <v>524</v>
@@ -5775,7 +5775,7 @@
         <v>25</v>
       </c>
       <c r="F126">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G126" t="s">
         <v>528</v>

</xml_diff>